<commit_message>
Programme v4.8: shorter tender, gateways, float and simple-job design; construction rows from test batch 4
TN1 8-10 wks up to 1,500 m2 (was 10-14), 10-12 above; GW / GW3 1 wk for
150-1,500 m2; PROG-FLOAT +1 wk per 26 (was 13); new DS2/3/4-DM and -EW rows
(read by typeDur); CN3 S4-S6 18-28 / 24-34 / 30-44; CN1 S6 50-70; CF1 S4
10-14; CX1 S1-S4 raised (10-14 ... 22-30), CX2 S2-S3 raised to stay above.
Edited through Excel COM; row-by-ID diff shows only these rows plus the
README version and changelog line.

Batch 4 offline: 28 of 30 programmes shorter; within 10% of the reviewer's
stage-by-stage figure 13 (was 7).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Estates_AI_Programme_v4_3.xlsx
+++ b/Estates_AI_Programme_v4_3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\estates-ai-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2EAA613-BD6D-414E-BC33-3C77CFA615CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8581785-52BB-4F5C-914A-43DBEE0B3F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="527">
   <si>
     <t>ESTATES AI TOOL — PROGRAMME DURATION REFERENCE</t>
   </si>
@@ -957,9 +957,6 @@
     <t>UPLIFT_PCT_RULE</t>
   </si>
   <si>
-    <t>+1 wk per 13 wks</t>
-  </si>
-  <si>
     <t>Always</t>
   </si>
   <si>
@@ -1554,13 +1551,64 @@
     <t>45-260</t>
   </si>
   <si>
-    <t>v4.7  ·  October 2026  ·  Nabil Kayali</t>
-  </si>
-  <si>
     <t>v4.7</t>
   </si>
   <si>
     <t>No duration changed. Numbers the app used to hold in its code now live here: size-band limits SB-S1…SB-S7 and the whole-programme sense-check envelopes PB-S1…PB-S7 on Modifiers. The app no longer has backup durations: it refuses a workbook missing SV3–SV6, PL1, PL3–PL5, BC1, TN1, TN2, CH1 or any SB / PB row, and it no longer picks a tender from the project value on its own (the Procurement Reference decides; before that step the programme uses TN1, marked provisional).</t>
+  </si>
+  <si>
+    <t>DS2-DM</t>
+  </si>
+  <si>
+    <t>Stage 2 — Concept (demolition only)</t>
+  </si>
+  <si>
+    <t>Used instead of the building row for this project type</t>
+  </si>
+  <si>
+    <t>v4.8 (test batch 4): a demolition or external works job has short design stages, not a building's.</t>
+  </si>
+  <si>
+    <t>DS3-DM</t>
+  </si>
+  <si>
+    <t>Stage 3 — Developed (demolition only)</t>
+  </si>
+  <si>
+    <t>DS4-DM</t>
+  </si>
+  <si>
+    <t>Stage 4 — Technical (demolition only)</t>
+  </si>
+  <si>
+    <t>DS2-EW</t>
+  </si>
+  <si>
+    <t>Stage 2 — Concept (external works only)</t>
+  </si>
+  <si>
+    <t>DS3-EW</t>
+  </si>
+  <si>
+    <t>Stage 3 — Developed (external works only)</t>
+  </si>
+  <si>
+    <t>DS4-EW</t>
+  </si>
+  <si>
+    <t>Stage 4 — Technical (external works only)</t>
+  </si>
+  <si>
+    <t>+1 wk per 26 wks</t>
+  </si>
+  <si>
+    <t>v4.8  ·  October 2026  ·  Nabil Kayali</t>
+  </si>
+  <si>
+    <t>v4.8</t>
+  </si>
+  <si>
+    <t>Durations shortened after test batch 4 (11 Oct 2026, 30 scenarios): formal tender TN1 8–10 wks up to 1,500 m² and 10–12 above (was 10–14); client gateways GW / GW3 1 wk for 150–1,500 m² (was 2); programme float PROG-FLOAT +1 wk per 26 (was 13); new design rows DS2/DS3/DS4-DM and -EW for demolition and external works only; construction CN3 industrial S4–S6 18–28 / 24–34 / 30–44 (was 22–36 / 32–52 / 48–72), CN1 S6 50–70 (was 60–84), CF1 S4 10–14 (was 12–20), CX1 single-storey extension S1–S4 10–14 / 14–20 / 18–24 / 22–30 (was 7–10 / 8–12 / 12–18 / 18–26), CX2 S2–S3 16–22 / 20–28 (was 12–18 / 18–26) so multi-storey stays above single-storey.</t>
   </si>
 </sst>
 </file>
@@ -2004,7 +2052,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -2022,7 +2070,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>508</v>
+        <v>524</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
@@ -2096,15 +2144,15 @@
         <v>17</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>412</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2124,7 +2172,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2172,7 +2220,7 @@
         <v>31</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
@@ -2317,34 +2365,42 @@
     </row>
     <row r="43" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>409</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>416</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>455</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>526</v>
       </c>
     </row>
   </sheetData>
@@ -2358,7 +2414,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:U37"/>
+  <dimension ref="A1:U43"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -3397,497 +3453,537 @@
         <v>132</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="14"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="14"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="14"/>
-      <c r="R18" s="14"/>
-      <c r="S18" s="14"/>
-      <c r="T18" s="14"/>
-      <c r="U18" s="15"/>
-    </row>
-    <row r="19" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="D18" s="7">
+        <v>1</v>
+      </c>
+      <c r="E18" s="7">
+        <v>1</v>
+      </c>
+      <c r="F18" s="7">
+        <v>1</v>
+      </c>
+      <c r="G18" s="7">
+        <v>2</v>
+      </c>
+      <c r="H18" s="7">
+        <v>1</v>
+      </c>
+      <c r="I18" s="7">
+        <v>2</v>
+      </c>
+      <c r="J18" s="7">
+        <v>1</v>
+      </c>
+      <c r="K18" s="7">
+        <v>2</v>
+      </c>
+      <c r="L18" s="7">
+        <v>2</v>
+      </c>
+      <c r="M18" s="7">
+        <v>3</v>
+      </c>
+      <c r="N18" s="7">
+        <v>2</v>
+      </c>
+      <c r="O18" s="7">
+        <v>3</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R18" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="S18" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="T18" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="U18" s="7" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>144</v>
+        <v>513</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>146</v>
+        <v>514</v>
       </c>
       <c r="D19" s="7">
         <v>1</v>
       </c>
       <c r="E19" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" s="7">
         <v>2</v>
       </c>
       <c r="G19" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H19" s="7">
         <v>2</v>
       </c>
       <c r="I19" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J19" s="7">
         <v>2</v>
       </c>
       <c r="K19" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L19" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M19" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N19" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P19" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="R19" s="7" t="s">
         <v>112</v>
       </c>
       <c r="S19" s="7" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="T19" s="7" t="s">
-        <v>148</v>
+        <v>511</v>
       </c>
       <c r="U19" s="7" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>150</v>
+        <v>515</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>151</v>
+        <v>516</v>
       </c>
       <c r="D20" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" s="7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20" s="7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H20" s="7">
         <v>2</v>
       </c>
       <c r="I20" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J20" s="7">
         <v>2</v>
       </c>
       <c r="K20" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L20" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M20" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N20" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P20" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q20" s="7" t="s">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="R20" s="7" t="s">
         <v>112</v>
       </c>
       <c r="S20" s="7" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="T20" s="7" t="s">
-        <v>152</v>
+        <v>511</v>
       </c>
       <c r="U20" s="7" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="14"/>
-      <c r="O21" s="14"/>
-      <c r="P21" s="14"/>
-      <c r="Q21" s="14"/>
-      <c r="R21" s="14"/>
-      <c r="S21" s="14"/>
-      <c r="T21" s="14"/>
-      <c r="U21" s="15"/>
-    </row>
-    <row r="22" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="D21" s="7">
+        <v>1</v>
+      </c>
+      <c r="E21" s="7">
+        <v>1</v>
+      </c>
+      <c r="F21" s="7">
+        <v>1</v>
+      </c>
+      <c r="G21" s="7">
+        <v>2</v>
+      </c>
+      <c r="H21" s="7">
+        <v>2</v>
+      </c>
+      <c r="I21" s="7">
+        <v>3</v>
+      </c>
+      <c r="J21" s="7">
+        <v>2</v>
+      </c>
+      <c r="K21" s="7">
+        <v>3</v>
+      </c>
+      <c r="L21" s="7">
+        <v>3</v>
+      </c>
+      <c r="M21" s="7">
+        <v>4</v>
+      </c>
+      <c r="N21" s="7">
+        <v>3</v>
+      </c>
+      <c r="O21" s="7">
+        <v>4</v>
+      </c>
+      <c r="P21" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="S21" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="T21" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="U21" s="7" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>155</v>
+        <v>519</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>156</v>
+        <v>109</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>157</v>
+        <v>520</v>
       </c>
       <c r="D22" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E22" s="7">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F22" s="7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G22" s="7">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H22" s="7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I22" s="7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J22" s="7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K22" s="7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="L22" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M22" s="7">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="N22" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O22" s="7">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P22" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>158</v>
+        <v>111</v>
       </c>
       <c r="R22" s="7" t="s">
-        <v>159</v>
+        <v>112</v>
       </c>
       <c r="S22" s="7" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="T22" s="7" t="s">
-        <v>160</v>
+        <v>511</v>
       </c>
       <c r="U22" s="7" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>162</v>
+        <v>521</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>156</v>
+        <v>109</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>163</v>
+        <v>522</v>
       </c>
       <c r="D23" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E23" s="7">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F23" s="7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G23" s="7">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H23" s="7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I23" s="7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J23" s="7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K23" s="7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="L23" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M23" s="7">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="N23" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O23" s="7">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="P23" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q23" s="7" t="s">
-        <v>158</v>
+        <v>111</v>
       </c>
       <c r="R23" s="7" t="s">
-        <v>159</v>
+        <v>112</v>
       </c>
       <c r="S23" s="7" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="T23" s="7" t="s">
-        <v>164</v>
+        <v>511</v>
       </c>
       <c r="U23" s="7" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="D24" s="7">
-        <v>4</v>
-      </c>
-      <c r="E24" s="7">
-        <v>8</v>
-      </c>
-      <c r="F24" s="7">
-        <v>4</v>
-      </c>
-      <c r="G24" s="7">
-        <v>8</v>
-      </c>
-      <c r="H24" s="7">
-        <v>4</v>
-      </c>
-      <c r="I24" s="7">
-        <v>8</v>
-      </c>
-      <c r="J24" s="7">
-        <v>4</v>
-      </c>
-      <c r="K24" s="7">
-        <v>8</v>
-      </c>
-      <c r="L24" s="7">
-        <v>4</v>
-      </c>
-      <c r="M24" s="7">
-        <v>8</v>
-      </c>
-      <c r="N24" s="7">
-        <v>4</v>
-      </c>
-      <c r="O24" s="7">
-        <v>8</v>
-      </c>
-      <c r="P24" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q24" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="R24" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="S24" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="T24" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="U24" s="7" t="s">
-        <v>169</v>
-      </c>
+        <v>512</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14"/>
+      <c r="M24" s="14"/>
+      <c r="N24" s="14"/>
+      <c r="O24" s="14"/>
+      <c r="P24" s="14"/>
+      <c r="Q24" s="14"/>
+      <c r="R24" s="14"/>
+      <c r="S24" s="14"/>
+      <c r="T24" s="14"/>
+      <c r="U24" s="15"/>
     </row>
     <row r="25" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>170</v>
+        <v>144</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="D25" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E25" s="7">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="F25" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G25" s="7">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="H25" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I25" s="7">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J25" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K25" s="7">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="L25" s="7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="M25" s="7">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="N25" s="7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O25" s="7">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="P25" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="R25" s="7" t="s">
-        <v>159</v>
+        <v>112</v>
       </c>
       <c r="S25" s="7" t="s">
         <v>83</v>
       </c>
       <c r="T25" s="7" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="U25" s="7" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>174</v>
+        <v>150</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>175</v>
+        <v>151</v>
       </c>
       <c r="D26" s="7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E26" s="7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F26" s="7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G26" s="7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H26" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I26" s="7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J26" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K26" s="7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L26" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M26" s="7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N26" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O26" s="7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="P26" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q26" s="7" t="s">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="R26" s="7" t="s">
         <v>112</v>
@@ -3896,302 +3992,342 @@
         <v>83</v>
       </c>
       <c r="T26" s="7" t="s">
-        <v>176</v>
+        <v>152</v>
       </c>
       <c r="U26" s="7" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="B27" s="6" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14"/>
+      <c r="L27" s="14"/>
+      <c r="M27" s="14"/>
+      <c r="N27" s="14"/>
+      <c r="O27" s="14"/>
+      <c r="P27" s="14"/>
+      <c r="Q27" s="14"/>
+      <c r="R27" s="14"/>
+      <c r="S27" s="14"/>
+      <c r="T27" s="14"/>
+      <c r="U27" s="15"/>
+    </row>
+    <row r="28" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="D27" s="7">
-        <v>0</v>
-      </c>
-      <c r="E27" s="7">
-        <v>0</v>
-      </c>
-      <c r="F27" s="7">
-        <v>0</v>
-      </c>
-      <c r="G27" s="7">
-        <v>0</v>
-      </c>
-      <c r="H27" s="7">
-        <v>0</v>
-      </c>
-      <c r="I27" s="7">
-        <v>0</v>
-      </c>
-      <c r="J27" s="7">
-        <v>0</v>
-      </c>
-      <c r="K27" s="7">
-        <v>0</v>
-      </c>
-      <c r="L27" s="7">
-        <v>0</v>
-      </c>
-      <c r="M27" s="7">
-        <v>0</v>
-      </c>
-      <c r="N27" s="7">
-        <v>0</v>
-      </c>
-      <c r="O27" s="7">
-        <v>0</v>
-      </c>
-      <c r="P27" s="7" t="s">
+      <c r="C28" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D28" s="7">
+        <v>8</v>
+      </c>
+      <c r="E28" s="7">
+        <v>13</v>
+      </c>
+      <c r="F28" s="7">
+        <v>8</v>
+      </c>
+      <c r="G28" s="7">
+        <v>13</v>
+      </c>
+      <c r="H28" s="7">
+        <v>8</v>
+      </c>
+      <c r="I28" s="7">
+        <v>13</v>
+      </c>
+      <c r="J28" s="7">
+        <v>8</v>
+      </c>
+      <c r="K28" s="7">
+        <v>13</v>
+      </c>
+      <c r="L28" s="7">
+        <v>8</v>
+      </c>
+      <c r="M28" s="7">
+        <v>13</v>
+      </c>
+      <c r="N28" s="7">
+        <v>8</v>
+      </c>
+      <c r="O28" s="7">
+        <v>13</v>
+      </c>
+      <c r="P28" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="Q27" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="R27" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="S27" s="7" t="s">
+      <c r="Q28" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="R28" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="S28" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="T27" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="U27" s="7" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
-        <v>183</v>
-      </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
-      <c r="L28" s="17"/>
-      <c r="M28" s="17"/>
-      <c r="N28" s="17"/>
-      <c r="O28" s="17"/>
-      <c r="P28" s="17"/>
-      <c r="Q28" s="17"/>
-      <c r="R28" s="17"/>
-      <c r="S28" s="17"/>
-      <c r="T28" s="17"/>
-      <c r="U28" s="18"/>
+      <c r="T28" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="U28" s="7" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="29" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="D29" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E29" s="7">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F29" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G29" s="7">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H29" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I29" s="7">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J29" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K29" s="7">
+        <v>13</v>
+      </c>
+      <c r="L29" s="7">
         <v>8</v>
       </c>
-      <c r="L29" s="7">
-        <v>5</v>
-      </c>
       <c r="M29" s="7">
+        <v>13</v>
+      </c>
+      <c r="N29" s="7">
         <v>8</v>
       </c>
-      <c r="N29" s="7">
-        <v>6</v>
-      </c>
       <c r="O29" s="7">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P29" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q29" s="7" t="s">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="R29" s="7" t="s">
-        <v>187</v>
+        <v>159</v>
       </c>
       <c r="S29" s="7" t="s">
         <v>83</v>
       </c>
       <c r="T29" s="7" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="U29" s="7" t="s">
-        <v>189</v>
+        <v>165</v>
       </c>
     </row>
     <row r="30" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>190</v>
+        <v>166</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>191</v>
+        <v>167</v>
       </c>
       <c r="D30" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F30" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G30" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H30" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I30" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J30" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K30" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L30" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M30" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N30" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O30" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P30" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q30" s="7" t="s">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="R30" s="7" t="s">
-        <v>187</v>
+        <v>159</v>
       </c>
       <c r="S30" s="7" t="s">
         <v>83</v>
       </c>
       <c r="T30" s="7" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="U30" s="7" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
-      <c r="M31" s="14"/>
-      <c r="N31" s="14"/>
-      <c r="O31" s="14"/>
-      <c r="P31" s="14"/>
-      <c r="Q31" s="14"/>
-      <c r="R31" s="14"/>
-      <c r="S31" s="14"/>
-      <c r="T31" s="14"/>
-      <c r="U31" s="15"/>
-    </row>
-    <row r="32" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D31" s="7">
+        <v>8</v>
+      </c>
+      <c r="E31" s="7">
+        <v>13</v>
+      </c>
+      <c r="F31" s="7">
+        <v>8</v>
+      </c>
+      <c r="G31" s="7">
+        <v>13</v>
+      </c>
+      <c r="H31" s="7">
+        <v>8</v>
+      </c>
+      <c r="I31" s="7">
+        <v>13</v>
+      </c>
+      <c r="J31" s="7">
+        <v>8</v>
+      </c>
+      <c r="K31" s="7">
+        <v>13</v>
+      </c>
+      <c r="L31" s="7">
+        <v>8</v>
+      </c>
+      <c r="M31" s="7">
+        <v>13</v>
+      </c>
+      <c r="N31" s="7">
+        <v>8</v>
+      </c>
+      <c r="O31" s="7">
+        <v>13</v>
+      </c>
+      <c r="P31" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q31" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="R31" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="S31" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="T31" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="U31" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>195</v>
+        <v>174</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>196</v>
+        <v>156</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>197</v>
+        <v>175</v>
       </c>
       <c r="D32" s="7">
+        <v>4</v>
+      </c>
+      <c r="E32" s="7">
         <v>6</v>
       </c>
-      <c r="E32" s="7">
-        <v>8</v>
-      </c>
       <c r="F32" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G32" s="7">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H32" s="7">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I32" s="7">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="J32" s="7">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K32" s="7">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="L32" s="7">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="M32" s="7">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="N32" s="7">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="O32" s="7">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="P32" s="7" t="s">
         <v>80</v>
@@ -4206,63 +4342,63 @@
         <v>83</v>
       </c>
       <c r="T32" s="7" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="U32" s="7" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
     </row>
     <row r="33" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>196</v>
+        <v>156</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="D33" s="7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E33" s="7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F33" s="7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G33" s="7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H33" s="7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I33" s="7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J33" s="7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K33" s="7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L33" s="7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M33" s="7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N33" s="7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O33" s="7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P33" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q33" s="7" t="s">
-        <v>111</v>
+        <v>180</v>
       </c>
       <c r="R33" s="7" t="s">
         <v>112</v>
@@ -4271,187 +4407,147 @@
         <v>83</v>
       </c>
       <c r="T33" s="7" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="U33" s="7" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D34" s="7">
-        <v>3</v>
-      </c>
-      <c r="E34" s="7">
-        <v>4</v>
-      </c>
-      <c r="F34" s="7">
-        <v>4</v>
-      </c>
-      <c r="G34" s="7">
-        <v>5</v>
-      </c>
-      <c r="H34" s="7">
-        <v>4</v>
-      </c>
-      <c r="I34" s="7">
-        <v>5</v>
-      </c>
-      <c r="J34" s="7">
-        <v>4</v>
-      </c>
-      <c r="K34" s="7">
-        <v>6</v>
-      </c>
-      <c r="L34" s="7">
-        <v>4</v>
-      </c>
-      <c r="M34" s="7">
-        <v>6</v>
-      </c>
-      <c r="N34" s="7">
-        <v>4</v>
-      </c>
-      <c r="O34" s="7">
-        <v>6</v>
-      </c>
-      <c r="P34" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q34" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="R34" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="S34" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="T34" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="U34" s="7" t="s">
-        <v>207</v>
-      </c>
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A34" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="17"/>
+      <c r="K34" s="17"/>
+      <c r="L34" s="17"/>
+      <c r="M34" s="17"/>
+      <c r="N34" s="17"/>
+      <c r="O34" s="17"/>
+      <c r="P34" s="17"/>
+      <c r="Q34" s="17"/>
+      <c r="R34" s="17"/>
+      <c r="S34" s="17"/>
+      <c r="T34" s="17"/>
+      <c r="U34" s="18"/>
     </row>
     <row r="35" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>426</v>
+        <v>184</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>427</v>
+        <v>186</v>
       </c>
       <c r="D35" s="7">
         <v>2</v>
       </c>
       <c r="E35" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F35" s="7">
         <v>2</v>
       </c>
       <c r="G35" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H35" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I35" s="7">
         <v>4</v>
       </c>
       <c r="J35" s="7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K35" s="7">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L35" s="7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M35" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N35" s="7">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O35" s="7">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="P35" s="7" t="s">
         <v>80</v>
       </c>
       <c r="Q35" s="7" t="s">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="R35" s="7" t="s">
-        <v>112</v>
+        <v>187</v>
       </c>
       <c r="S35" s="7" t="s">
         <v>83</v>
       </c>
       <c r="T35" s="7" t="s">
-        <v>428</v>
+        <v>188</v>
       </c>
       <c r="U35" s="7" t="s">
-        <v>429</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>400</v>
+        <v>190</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>78</v>
+        <v>185</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>401</v>
+        <v>191</v>
       </c>
       <c r="D36" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F36" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G36" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H36" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I36" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J36" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L36" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M36" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N36" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O36" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P36" s="7" t="s">
         <v>80</v>
@@ -4460,91 +4556,441 @@
         <v>81</v>
       </c>
       <c r="R36" s="7" t="s">
-        <v>82</v>
+        <v>187</v>
       </c>
       <c r="S36" s="7" t="s">
         <v>83</v>
       </c>
       <c r="T36" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="U36" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A37" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="14"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14"/>
+      <c r="L37" s="14"/>
+      <c r="M37" s="14"/>
+      <c r="N37" s="14"/>
+      <c r="O37" s="14"/>
+      <c r="P37" s="14"/>
+      <c r="Q37" s="14"/>
+      <c r="R37" s="14"/>
+      <c r="S37" s="14"/>
+      <c r="T37" s="14"/>
+      <c r="U37" s="15"/>
+    </row>
+    <row r="38" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="D38" s="7">
+        <v>6</v>
+      </c>
+      <c r="E38" s="7">
+        <v>8</v>
+      </c>
+      <c r="F38" s="7">
+        <v>8</v>
+      </c>
+      <c r="G38" s="7">
+        <v>10</v>
+      </c>
+      <c r="H38" s="7">
+        <v>8</v>
+      </c>
+      <c r="I38" s="7">
+        <v>10</v>
+      </c>
+      <c r="J38" s="7">
+        <v>8</v>
+      </c>
+      <c r="K38" s="7">
+        <v>10</v>
+      </c>
+      <c r="L38" s="7">
+        <v>10</v>
+      </c>
+      <c r="M38" s="7">
+        <v>12</v>
+      </c>
+      <c r="N38" s="7">
+        <v>10</v>
+      </c>
+      <c r="O38" s="7">
+        <v>12</v>
+      </c>
+      <c r="P38" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q38" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R38" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="S38" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="T38" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="U38" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D39" s="7">
+        <v>3</v>
+      </c>
+      <c r="E39" s="7">
+        <v>4</v>
+      </c>
+      <c r="F39" s="7">
+        <v>3</v>
+      </c>
+      <c r="G39" s="7">
+        <v>4</v>
+      </c>
+      <c r="H39" s="7">
+        <v>4</v>
+      </c>
+      <c r="I39" s="7">
+        <v>6</v>
+      </c>
+      <c r="J39" s="7">
+        <v>4</v>
+      </c>
+      <c r="K39" s="7">
+        <v>6</v>
+      </c>
+      <c r="L39" s="7">
+        <v>4</v>
+      </c>
+      <c r="M39" s="7">
+        <v>6</v>
+      </c>
+      <c r="N39" s="7">
+        <v>4</v>
+      </c>
+      <c r="O39" s="7">
+        <v>6</v>
+      </c>
+      <c r="P39" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q39" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R39" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="S39" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="T39" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D40" s="7">
+        <v>3</v>
+      </c>
+      <c r="E40" s="7">
+        <v>4</v>
+      </c>
+      <c r="F40" s="7">
+        <v>4</v>
+      </c>
+      <c r="G40" s="7">
+        <v>5</v>
+      </c>
+      <c r="H40" s="7">
+        <v>4</v>
+      </c>
+      <c r="I40" s="7">
+        <v>5</v>
+      </c>
+      <c r="J40" s="7">
+        <v>4</v>
+      </c>
+      <c r="K40" s="7">
+        <v>6</v>
+      </c>
+      <c r="L40" s="7">
+        <v>4</v>
+      </c>
+      <c r="M40" s="7">
+        <v>6</v>
+      </c>
+      <c r="N40" s="7">
+        <v>4</v>
+      </c>
+      <c r="O40" s="7">
+        <v>6</v>
+      </c>
+      <c r="P40" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q40" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R40" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="S40" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="T40" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="U40" s="7" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="D41" s="7">
+        <v>2</v>
+      </c>
+      <c r="E41" s="7">
+        <v>3</v>
+      </c>
+      <c r="F41" s="7">
+        <v>2</v>
+      </c>
+      <c r="G41" s="7">
+        <v>3</v>
+      </c>
+      <c r="H41" s="7">
+        <v>3</v>
+      </c>
+      <c r="I41" s="7">
+        <v>4</v>
+      </c>
+      <c r="J41" s="7">
+        <v>3</v>
+      </c>
+      <c r="K41" s="7">
+        <v>4</v>
+      </c>
+      <c r="L41" s="7">
+        <v>3</v>
+      </c>
+      <c r="M41" s="7">
+        <v>5</v>
+      </c>
+      <c r="N41" s="7">
+        <v>3</v>
+      </c>
+      <c r="O41" s="7">
+        <v>5</v>
+      </c>
+      <c r="P41" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q41" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R41" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="S41" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="T41" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="U41" s="7" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="42" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="D42" s="7">
+        <v>2</v>
+      </c>
+      <c r="E42" s="7">
+        <v>4</v>
+      </c>
+      <c r="F42" s="7">
+        <v>2</v>
+      </c>
+      <c r="G42" s="7">
+        <v>4</v>
+      </c>
+      <c r="H42" s="7">
+        <v>2</v>
+      </c>
+      <c r="I42" s="7">
+        <v>4</v>
+      </c>
+      <c r="J42" s="7">
+        <v>2</v>
+      </c>
+      <c r="K42" s="7">
+        <v>4</v>
+      </c>
+      <c r="L42" s="7">
+        <v>2</v>
+      </c>
+      <c r="M42" s="7">
+        <v>4</v>
+      </c>
+      <c r="N42" s="7">
+        <v>2</v>
+      </c>
+      <c r="O42" s="7">
+        <v>4</v>
+      </c>
+      <c r="P42" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q42" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="R42" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="S42" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="T42" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="U42" s="7" t="s">
         <v>402</v>
       </c>
-      <c r="U36" s="7" t="s">
+    </row>
+    <row r="43" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="37" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
+      <c r="B43" s="6" t="s">
         <v>404</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="C43" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="D43" s="7">
+        <v>12</v>
+      </c>
+      <c r="E43" s="7">
+        <v>24</v>
+      </c>
+      <c r="F43" s="7">
+        <v>12</v>
+      </c>
+      <c r="G43" s="7">
+        <v>24</v>
+      </c>
+      <c r="H43" s="7">
+        <v>12</v>
+      </c>
+      <c r="I43" s="7">
+        <v>24</v>
+      </c>
+      <c r="J43" s="7">
+        <v>12</v>
+      </c>
+      <c r="K43" s="7">
+        <v>24</v>
+      </c>
+      <c r="L43" s="7">
+        <v>12</v>
+      </c>
+      <c r="M43" s="7">
+        <v>24</v>
+      </c>
+      <c r="N43" s="7">
+        <v>12</v>
+      </c>
+      <c r="O43" s="7">
+        <v>24</v>
+      </c>
+      <c r="P43" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q43" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R43" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="S43" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="T43" s="7" t="s">
         <v>406</v>
       </c>
-      <c r="D37" s="7">
-        <v>12</v>
-      </c>
-      <c r="E37" s="7">
-        <v>24</v>
-      </c>
-      <c r="F37" s="7">
-        <v>12</v>
-      </c>
-      <c r="G37" s="7">
-        <v>24</v>
-      </c>
-      <c r="H37" s="7">
-        <v>12</v>
-      </c>
-      <c r="I37" s="7">
-        <v>24</v>
-      </c>
-      <c r="J37" s="7">
-        <v>12</v>
-      </c>
-      <c r="K37" s="7">
-        <v>24</v>
-      </c>
-      <c r="L37" s="7">
-        <v>12</v>
-      </c>
-      <c r="M37" s="7">
-        <v>24</v>
-      </c>
-      <c r="N37" s="7">
-        <v>12</v>
-      </c>
-      <c r="O37" s="7">
-        <v>24</v>
-      </c>
-      <c r="P37" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q37" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="R37" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="S37" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="T37" s="7" t="s">
+      <c r="U43" s="7" t="s">
         <v>407</v>
-      </c>
-      <c r="U37" s="7" t="s">
-        <v>408</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A31:U31"/>
+    <mergeCell ref="A37:U37"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A9:U9"/>
-    <mergeCell ref="A18:U18"/>
-    <mergeCell ref="A21:U21"/>
-    <mergeCell ref="A28:U28"/>
+    <mergeCell ref="A24:U24"/>
+    <mergeCell ref="A27:U27"/>
+    <mergeCell ref="A34:U34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4606,10 +5052,10 @@
         <v>69</v>
       </c>
       <c r="O1" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="P1" s="5" t="s">
         <v>418</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>419</v>
       </c>
       <c r="Q1" s="5" t="s">
         <v>70</v>
@@ -4656,10 +5102,10 @@
         <v>64</v>
       </c>
       <c r="M2" s="7">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="N2" s="7">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="Q2" s="7" t="s">
         <v>80</v>
@@ -4744,22 +5190,22 @@
         <v>22</v>
       </c>
       <c r="I4" s="7">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J4" s="7">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="K4" s="7">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="L4" s="7">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="M4" s="7">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="N4" s="7">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="Q4" s="7" t="s">
         <v>80</v>
@@ -4776,28 +5222,28 @@
         <v>220</v>
       </c>
       <c r="C5" s="6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D5" s="7">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E5" s="7">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F5" s="7">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="G5" s="7">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H5" s="7">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="I5" s="7">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J5" s="7">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
@@ -4824,16 +5270,16 @@
         <v>14</v>
       </c>
       <c r="E6" s="7">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F6" s="7">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G6" s="7">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H6" s="7">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I6" s="7">
         <v>26</v>
@@ -4913,7 +5359,7 @@
         <v>80</v>
       </c>
       <c r="R7" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
@@ -4992,10 +5438,10 @@
         <v>12</v>
       </c>
       <c r="I9" s="7">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J9" s="7">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="K9" s="7">
         <v>20</v>
@@ -5063,7 +5509,7 @@
         <v>80</v>
       </c>
       <c r="R10" s="7" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
@@ -5263,7 +5709,7 @@
         <v>80</v>
       </c>
       <c r="R14" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -5443,7 +5889,7 @@
         <v>276</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5466,7 +5912,7 @@
         <v>279</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5512,7 +5958,7 @@
         <v>286</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
@@ -5578,7 +6024,7 @@
         <v>0.1</v>
       </c>
       <c r="F13" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="G13" t="s">
         <v>302</v>
@@ -5601,10 +6047,10 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="F14" t="s">
+        <v>430</v>
+      </c>
+      <c r="G14" t="s">
         <v>431</v>
-      </c>
-      <c r="G14" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="24" x14ac:dyDescent="0.25">
@@ -5621,450 +6067,450 @@
         <v>308</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="F15" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="G15" s="6" t="s">
         <v>310</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="10" t="s">
         <v>436</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G16" s="6" t="s">
         <v>438</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>440</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="C17" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>441</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>442</v>
-      </c>
       <c r="F17" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="G17" s="6" t="s">
         <v>438</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>444</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>445</v>
-      </c>
       <c r="F18" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>438</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="C19" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>447</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>448</v>
-      </c>
       <c r="F19" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="G19" s="6" t="s">
         <v>438</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>450</v>
       </c>
-      <c r="C20" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>451</v>
-      </c>
       <c r="F20" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="G20" s="6" t="s">
         <v>438</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E21" s="10" t="s">
         <v>453</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>454</v>
-      </c>
       <c r="F21" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="G21" s="6" t="s">
         <v>438</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="36" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="C22" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>459</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="E22" s="10" t="s">
         <v>460</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="F22" s="6" t="s">
         <v>461</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="G22" s="6" t="s">
         <v>462</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>464</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E23" s="10" t="s">
         <v>465</v>
       </c>
-      <c r="C23" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="E23" s="10" t="s">
+      <c r="F23" s="6" t="s">
         <v>466</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>467</v>
       </c>
       <c r="G23" s="6"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>468</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E24" s="10" t="s">
         <v>469</v>
       </c>
-      <c r="C24" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>470</v>
-      </c>
       <c r="F24" s="6" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G24" s="6"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>471</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E25" s="10" t="s">
         <v>472</v>
       </c>
-      <c r="C25" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>473</v>
-      </c>
       <c r="F25" s="6" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G25" s="6"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="B26" s="6" t="s">
         <v>474</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="C26" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E26" s="10" t="s">
         <v>475</v>
       </c>
-      <c r="C26" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>476</v>
-      </c>
       <c r="F26" s="6" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G26" s="6"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>477</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E27" s="10" t="s">
         <v>478</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>479</v>
-      </c>
       <c r="F27" s="6" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G27" s="6"/>
     </row>
     <row r="28" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>480</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="C28" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E28" s="10" t="s">
         <v>481</v>
       </c>
-      <c r="C28" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="E28" s="10" t="s">
+      <c r="F28" s="6" t="s">
+        <v>466</v>
+      </c>
+      <c r="G28" s="6" t="s">
         <v>482</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>467</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="C29" s="6" t="s">
         <v>485</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="D29" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="E29" s="10" t="s">
         <v>487</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="F29" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="G29" s="6" t="s">
         <v>488</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>458</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="C30" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E30" s="10" t="s">
         <v>491</v>
       </c>
-      <c r="C30" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>492</v>
-      </c>
       <c r="F30" s="6" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G30" s="6"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>493</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E31" s="10" t="s">
         <v>494</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>495</v>
-      </c>
       <c r="F31" s="6" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="G31" s="6"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="B32" s="6" t="s">
         <v>496</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="C32" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E32" s="10" t="s">
         <v>497</v>
       </c>
-      <c r="C32" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>498</v>
-      </c>
       <c r="F32" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="G32" s="6"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>499</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="C33" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E33" s="10" t="s">
         <v>500</v>
       </c>
-      <c r="C33" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>501</v>
-      </c>
       <c r="F33" s="6" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="G33" s="6"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="C34" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E34" s="10" t="s">
         <v>503</v>
       </c>
-      <c r="C34" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>504</v>
-      </c>
       <c r="F34" s="6" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="G34" s="6"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="B35" s="6" t="s">
         <v>505</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="C35" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E35" s="10" t="s">
         <v>506</v>
       </c>
-      <c r="C35" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>507</v>
-      </c>
       <c r="F35" s="6" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="G35" s="6"/>
     </row>
@@ -6089,222 +6535,222 @@
   <sheetData>
     <row r="1" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>316</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>322</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>328</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>334</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>340</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>346</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>352</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>358</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>344</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>363</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>365</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>366</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>181</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>368</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="F11" s="6" t="s">
         <v>373</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>334</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -6327,103 +6773,103 @@
         <v>5</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>376</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
+        <v>377</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>378</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>380</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>382</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>384</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>386</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
+        <v>387</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>388</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>390</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>392</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>394</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>396</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>398</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>399</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Programme v4.10: durations reviewed against the owner's projects; M&E threshold moved to the workbook
Occupation uplift OCC-1 +15% (was 30%), OCC-2 +10% (was 20%) - Lakeside
occupied ran about 10% slower than vacant Riley Court; Claycroft now 73
weeks against 74 planned (was 82). DS3a 1 week, DS4a 1-2 (fired on almost
every project). Planning PL1/PL4 8-10 minor, 10-13 major; PL2 8-10 up to
1,500 m2. TN1 S1-S3 4-6/5-7/6-8. CF2 and CF1 S5-S6, CN1 S5, CN2 S3-S6,
CE1 S5-S6 shortened. Unchanged and confirmed: CR1, CD1, CF2 S1-S4, CH1.

The '4 or more services items' threshold for the design uplifts was a
number in the code; it is now Modifiers ME-HEAVY (4) and a required row.

Batch 4: 26 of 30 programmes shorter, none longer. 734 Vitest pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Estates_AI_Programme_v4_3.xlsx
+++ b/Estates_AI_Programme_v4_3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\estates-ai-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8D549F-5038-43EE-9AFB-2B8C33C7EA93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB5A6E9-E8C2-43C7-A44C-EE0134690F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2250" yWindow="2250" windowWidth="21600" windowHeight="11295" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="608">
   <si>
     <t>ESTATES AI TOOL — PROGRAMME DURATION REFERENCE</t>
   </si>
@@ -1624,9 +1624,6 @@
     <t>Healthcare</t>
   </si>
   <si>
-    <t>v4.9  ·  October 2026  ·  Nabil Kayali</t>
-  </si>
-  <si>
     <t>v4.9</t>
   </si>
   <si>
@@ -1829,6 +1826,33 @@
   </si>
   <si>
     <t>Site work restrictions (Q4.2a / Q4.2b, 11 Oct 2026): new sheet 'Restrictions' lists the periods a user can tick when work on site is not permitted, by building use (Education 6, Healthcare 2, Retail 3, Hospitality 2, Residential 1, Student accommodation 2, Industrial 1, Mixed use 1). Columns: ID, Building uses (Q1.3 labels, ';'), Restriction and Dates shown (what the user reads), Blocked periods (MM-DD/MM-DD, ';', repeated every year; a period may cross the new year), Notes. The user can also enter up to three specific date ranges. Construction is fitted around every ticked period. Add or change an option here; no code change.</t>
+  </si>
+  <si>
+    <t>ME-HEAVY</t>
+  </si>
+  <si>
+    <t>M&amp;E-heavy design uplift threshold</t>
+  </si>
+  <si>
+    <t>Stage 3 / Stage 4 design</t>
+  </si>
+  <si>
+    <t>THRESHOLD</t>
+  </si>
+  <si>
+    <t>Number of services (Group 5) items in Q2.3 at or above which DS3a and DS4a are added</t>
+  </si>
+  <si>
+    <t>Moved from the code (v4.10). DS3a / DS4a are now 1–2 weeks, so the threshold matters less.</t>
+  </si>
+  <si>
+    <t>v4.10  ·  October 2026  ·  Nabil Kayali</t>
+  </si>
+  <si>
+    <t>v4.10</t>
+  </si>
+  <si>
+    <t>Duration review against the owner's projects (11 Oct 2026). Occupation uplift OCC-1 +15% (was 30%), OCC-2 +10% (was 20%): Lakeside occupied ran about 10% slower than vacant Riley Court; Claycroft now 73 weeks against 74 planned. Design uplifts DS3a 1 week, DS4a 1 up to 500 m² and 2 above (were up to 3 and 4; they fired on almost every project). Planning PL1 / PL4 8–10 up to 1,500 m² (minor, 8-week statutory) and 10–13 above (major); PL2 8–10 up to 1,500 m². Tender TN1 S1–S3 4–6 / 5–7 / 6–8. Construction CF2 S5–S6 12–18 / 18–28, CF1 S5–S6 16–24 / 24–36, CN1 S5 40–56, CN2 S3–S6 26–38 / 36–52 / 50–70 / 70–95, CE1 S5–S6 8–12 / 10–16. New Modifiers row ME-HEAVY (4) holds the threshold the code used. Unchanged and confirmed: CR1 (Riley Court 41 vs 42), CD1 (Whitefields 14), CF2 S1–S4 (Co-op 8 vs 7, IBRB 3), CH1.</t>
   </si>
 </sst>
 </file>
@@ -2006,6 +2030,11 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2027,11 +2056,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2297,7 +2321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -2305,17 +2329,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
+      <c r="B1" s="15"/>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>531</v>
+        <v>605</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
@@ -2650,10 +2674,18 @@
     </row>
     <row r="48" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>607</v>
       </c>
     </row>
   </sheetData>
@@ -2747,29 +2779,29 @@
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
-      <c r="U2" s="15"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="18"/>
     </row>
     <row r="3" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -3162,29 +3194,29 @@
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="14"/>
-      <c r="M9" s="14"/>
-      <c r="N9" s="14"/>
-      <c r="O9" s="14"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="14"/>
-      <c r="R9" s="14"/>
-      <c r="S9" s="14"/>
-      <c r="T9" s="14"/>
-      <c r="U9" s="15"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
+      <c r="M9" s="17"/>
+      <c r="N9" s="17"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+      <c r="S9" s="17"/>
+      <c r="T9" s="17"/>
+      <c r="U9" s="18"/>
     </row>
     <row r="10" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
@@ -3463,34 +3495,34 @@
         <v>1</v>
       </c>
       <c r="F14" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I14" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M14" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O14" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P14" s="7" t="s">
         <v>80</v>
@@ -3658,34 +3690,34 @@
         <v>1</v>
       </c>
       <c r="F17" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H17" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I17" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L17" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M17" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N17" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O17" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P17" s="7" t="s">
         <v>80</v>
@@ -4097,29 +4129,29 @@
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
-      <c r="Q24" s="14"/>
-      <c r="R24" s="14"/>
-      <c r="S24" s="14"/>
-      <c r="T24" s="14"/>
-      <c r="U24" s="15"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="17"/>
+      <c r="S24" s="17"/>
+      <c r="T24" s="17"/>
+      <c r="U24" s="18"/>
     </row>
     <row r="25" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
@@ -4252,29 +4284,29 @@
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="14"/>
-      <c r="M27" s="14"/>
-      <c r="N27" s="14"/>
-      <c r="O27" s="14"/>
-      <c r="P27" s="14"/>
-      <c r="Q27" s="14"/>
-      <c r="R27" s="14"/>
-      <c r="S27" s="14"/>
-      <c r="T27" s="14"/>
-      <c r="U27" s="15"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="17"/>
+      <c r="O27" s="17"/>
+      <c r="P27" s="17"/>
+      <c r="Q27" s="17"/>
+      <c r="R27" s="17"/>
+      <c r="S27" s="17"/>
+      <c r="T27" s="17"/>
+      <c r="U27" s="18"/>
     </row>
     <row r="28" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
@@ -4290,34 +4322,34 @@
         <v>8</v>
       </c>
       <c r="E28" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F28" s="7">
         <v>8</v>
       </c>
       <c r="G28" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H28" s="7">
         <v>8</v>
       </c>
       <c r="I28" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J28" s="7">
         <v>8</v>
       </c>
       <c r="K28" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L28" s="7">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M28" s="7">
         <v>13</v>
       </c>
       <c r="N28" s="7">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O28" s="7">
         <v>13</v>
@@ -4355,25 +4387,25 @@
         <v>8</v>
       </c>
       <c r="E29" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F29" s="7">
         <v>8</v>
       </c>
       <c r="G29" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H29" s="7">
         <v>8</v>
       </c>
       <c r="I29" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J29" s="7">
         <v>8</v>
       </c>
       <c r="K29" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L29" s="7">
         <v>8</v>
@@ -4485,34 +4517,34 @@
         <v>8</v>
       </c>
       <c r="E31" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F31" s="7">
         <v>8</v>
       </c>
       <c r="G31" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H31" s="7">
         <v>8</v>
       </c>
       <c r="I31" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J31" s="7">
         <v>8</v>
       </c>
       <c r="K31" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L31" s="7">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M31" s="7">
         <v>13</v>
       </c>
       <c r="N31" s="7">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O31" s="7">
         <v>13</v>
@@ -4667,29 +4699,29 @@
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="17"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="17"/>
-      <c r="K34" s="17"/>
-      <c r="L34" s="17"/>
-      <c r="M34" s="17"/>
-      <c r="N34" s="17"/>
-      <c r="O34" s="17"/>
-      <c r="P34" s="17"/>
-      <c r="Q34" s="17"/>
-      <c r="R34" s="17"/>
-      <c r="S34" s="17"/>
-      <c r="T34" s="17"/>
-      <c r="U34" s="18"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="20"/>
+      <c r="J34" s="20"/>
+      <c r="K34" s="20"/>
+      <c r="L34" s="20"/>
+      <c r="M34" s="20"/>
+      <c r="N34" s="20"/>
+      <c r="O34" s="20"/>
+      <c r="P34" s="20"/>
+      <c r="Q34" s="20"/>
+      <c r="R34" s="20"/>
+      <c r="S34" s="20"/>
+      <c r="T34" s="20"/>
+      <c r="U34" s="21"/>
     </row>
     <row r="35" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
@@ -4822,29 +4854,29 @@
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A37" s="13" t="s">
+      <c r="A37" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="14"/>
-      <c r="K37" s="14"/>
-      <c r="L37" s="14"/>
-      <c r="M37" s="14"/>
-      <c r="N37" s="14"/>
-      <c r="O37" s="14"/>
-      <c r="P37" s="14"/>
-      <c r="Q37" s="14"/>
-      <c r="R37" s="14"/>
-      <c r="S37" s="14"/>
-      <c r="T37" s="14"/>
-      <c r="U37" s="15"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17"/>
+      <c r="M37" s="17"/>
+      <c r="N37" s="17"/>
+      <c r="O37" s="17"/>
+      <c r="P37" s="17"/>
+      <c r="Q37" s="17"/>
+      <c r="R37" s="17"/>
+      <c r="S37" s="17"/>
+      <c r="T37" s="17"/>
+      <c r="U37" s="18"/>
     </row>
     <row r="38" spans="1:21" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
@@ -4857,22 +4889,22 @@
         <v>197</v>
       </c>
       <c r="D38" s="7">
+        <v>4</v>
+      </c>
+      <c r="E38" s="7">
         <v>6</v>
       </c>
-      <c r="E38" s="7">
+      <c r="F38" s="7">
+        <v>5</v>
+      </c>
+      <c r="G38" s="7">
+        <v>7</v>
+      </c>
+      <c r="H38" s="7">
+        <v>6</v>
+      </c>
+      <c r="I38" s="7">
         <v>8</v>
-      </c>
-      <c r="F38" s="7">
-        <v>8</v>
-      </c>
-      <c r="G38" s="7">
-        <v>10</v>
-      </c>
-      <c r="H38" s="7">
-        <v>8</v>
-      </c>
-      <c r="I38" s="7">
-        <v>10</v>
       </c>
       <c r="J38" s="7">
         <v>8</v>
@@ -5349,10 +5381,10 @@
         <v>48</v>
       </c>
       <c r="K2" s="7">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="L2" s="7">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="M2" s="7">
         <v>50</v>
@@ -5387,28 +5419,28 @@
         <v>32</v>
       </c>
       <c r="G3" s="7">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="H3" s="7">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="I3" s="7">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="J3" s="7">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="K3" s="7">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="L3" s="7">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="M3" s="7">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="N3" s="7">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="Q3" s="7" t="s">
         <v>80</v>
@@ -5697,16 +5729,16 @@
         <v>14</v>
       </c>
       <c r="K9" s="7">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L9" s="7">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="M9" s="7">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="N9" s="7">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="Q9" s="7" t="s">
         <v>80</v>
@@ -5747,16 +5779,16 @@
         <v>9</v>
       </c>
       <c r="K10" s="7">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="L10" s="7">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="M10" s="7">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="N10" s="7">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="Q10" s="7" t="s">
         <v>80</v>
@@ -5847,16 +5879,16 @@
         <v>10</v>
       </c>
       <c r="K12" s="7">
+        <v>8</v>
+      </c>
+      <c r="L12" s="7">
+        <v>12</v>
+      </c>
+      <c r="M12" s="7">
         <v>10</v>
       </c>
-      <c r="L12" s="7">
+      <c r="N12" s="7">
         <v>16</v>
-      </c>
-      <c r="M12" s="7">
-        <v>14</v>
-      </c>
-      <c r="N12" s="7">
-        <v>22</v>
       </c>
       <c r="Q12" s="7" t="s">
         <v>80</v>
@@ -5973,7 +6005,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -6136,7 +6168,7 @@
         <v>275</v>
       </c>
       <c r="E7" s="6">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>276</v>
@@ -6159,7 +6191,7 @@
         <v>275</v>
       </c>
       <c r="E8" s="6">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>279</v>
@@ -6193,102 +6225,102 @@
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="E10" s="6">
+        <v>4</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B11" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E11" s="6">
         <v>0.15</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G11" s="6" t="s">
         <v>424</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>288</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>289</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>291</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>292</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B13" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C13" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E13" s="6">
         <v>0</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G13" s="6" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="14" spans="1:7" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>300</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>301</v>
-      </c>
-      <c r="C13" t="s">
-        <v>274</v>
-      </c>
-      <c r="D13" t="s">
-        <v>275</v>
-      </c>
-      <c r="E13">
-        <v>0.1</v>
-      </c>
-      <c r="F13" t="s">
-        <v>429</v>
-      </c>
-      <c r="G13" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>303</v>
-      </c>
-      <c r="B14" t="s">
-        <v>304</v>
       </c>
       <c r="C14" t="s">
         <v>274</v>
@@ -6297,67 +6329,67 @@
         <v>275</v>
       </c>
       <c r="E14">
+        <v>0.1</v>
+      </c>
+      <c r="F14" t="s">
+        <v>429</v>
+      </c>
+      <c r="G14" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>303</v>
+      </c>
+      <c r="B15" t="s">
+        <v>304</v>
+      </c>
+      <c r="C15" t="s">
+        <v>274</v>
+      </c>
+      <c r="D15" t="s">
+        <v>275</v>
+      </c>
+      <c r="E15">
         <v>0.17499999999999999</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F15" t="s">
         <v>430</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G15" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+    <row r="16" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B16" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>523</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="G16" s="6" t="s">
         <v>310</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="48" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>432</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>433</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>436</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>439</v>
+        <v>432</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>440</v>
+        <v>433</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>434</v>
@@ -6366,7 +6398,7 @@
         <v>435</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>437</v>
@@ -6377,10 +6409,10 @@
     </row>
     <row r="18" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>434</v>
@@ -6389,7 +6421,7 @@
         <v>435</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>437</v>
@@ -6400,10 +6432,10 @@
     </row>
     <row r="19" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>434</v>
@@ -6412,7 +6444,7 @@
         <v>435</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>437</v>
@@ -6423,10 +6455,10 @@
     </row>
     <row r="20" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>434</v>
@@ -6435,7 +6467,7 @@
         <v>435</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>437</v>
@@ -6446,10 +6478,10 @@
     </row>
     <row r="21" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>434</v>
@@ -6458,7 +6490,7 @@
         <v>435</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>437</v>
@@ -6467,35 +6499,35 @@
         <v>438</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="36" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="48" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>453</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="36" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B23" s="6" t="s">
         <v>457</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>458</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>460</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>463</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>464</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>458</v>
@@ -6504,19 +6536,21 @@
         <v>459</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>466</v>
-      </c>
-      <c r="G23" s="6"/>
+        <v>461</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>462</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>458</v>
@@ -6525,7 +6559,7 @@
         <v>459</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>466</v>
@@ -6534,10 +6568,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>458</v>
@@ -6546,7 +6580,7 @@
         <v>459</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="F25" s="6" t="s">
         <v>466</v>
@@ -6555,10 +6589,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>458</v>
@@ -6567,7 +6601,7 @@
         <v>459</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>466</v>
@@ -6576,10 +6610,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>458</v>
@@ -6588,19 +6622,19 @@
         <v>459</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>466</v>
       </c>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>458</v>
@@ -6609,44 +6643,42 @@
         <v>459</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>466</v>
       </c>
-      <c r="G28" s="6" t="s">
+      <c r="G28" s="6"/>
+    </row>
+    <row r="29" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>481</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>466</v>
+      </c>
+      <c r="G29" s="6" t="s">
         <v>482</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="48" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+    <row r="30" spans="1:7" ht="48" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B30" s="6" t="s">
         <v>484</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>485</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>487</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>457</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>490</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>485</v>
@@ -6655,19 +6687,21 @@
         <v>486</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>464</v>
-      </c>
-      <c r="G30" s="6"/>
+        <v>457</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>485</v>
@@ -6676,19 +6710,19 @@
         <v>486</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="G31" s="6"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>485</v>
@@ -6697,19 +6731,19 @@
         <v>486</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="G32" s="6"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>485</v>
@@ -6718,19 +6752,19 @@
         <v>486</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="G33" s="6"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>485</v>
@@ -6739,19 +6773,19 @@
         <v>486</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="G34" s="6"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>485</v>
@@ -6760,12 +6794,33 @@
         <v>486</v>
       </c>
       <c r="E35" s="10" t="s">
+        <v>503</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="G35" s="6"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E36" s="10" t="s">
         <v>506</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="F36" s="6" t="s">
         <v>480</v>
       </c>
-      <c r="G35" s="6"/>
+      <c r="G36" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6787,268 +6842,268 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="11" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>533</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="20" t="s">
+      <c r="C3" s="12" t="s">
         <v>534</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="D3" s="12" t="s">
         <v>535</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="E3" s="12" t="s">
         <v>536</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="F3" s="12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>537</v>
       </c>
-      <c r="F3" s="20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+      <c r="B4" s="13" t="s">
+        <v>527</v>
+      </c>
+      <c r="C4" s="13" t="s">
         <v>538</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="D4" s="13" t="s">
+        <v>539</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>526</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>541</v>
+      </c>
+      <c r="B5" s="13" t="s">
         <v>527</v>
       </c>
-      <c r="C4" s="21" t="s">
-        <v>539</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>540</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>526</v>
-      </c>
-      <c r="F4" s="21" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+      <c r="C5" s="13" t="s">
         <v>542</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="D5" s="13" t="s">
+        <v>543</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>544</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>546</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>528</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>547</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>548</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>549</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>551</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>527</v>
       </c>
-      <c r="C5" s="21" t="s">
-        <v>543</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>544</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>545</v>
-      </c>
-      <c r="F5" s="21" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
-        <v>547</v>
-      </c>
-      <c r="B6" s="21" t="s">
+      <c r="C7" s="13" t="s">
+        <v>552</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>554</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>556</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>527</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>558</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>559</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>561</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>528</v>
       </c>
-      <c r="C6" s="21" t="s">
-        <v>548</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>549</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>550</v>
-      </c>
-      <c r="F6" s="21" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
-        <v>552</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>527</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>553</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>554</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>555</v>
-      </c>
-      <c r="F7" s="21" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>557</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>527</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>558</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>559</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>560</v>
-      </c>
-      <c r="F8" s="21" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
+      <c r="C9" s="13" t="s">
         <v>562</v>
       </c>
-      <c r="B9" s="21" t="s">
-        <v>528</v>
-      </c>
-      <c r="C9" s="21" t="s">
+      <c r="D9" s="13" t="s">
         <v>563</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="E9" s="13" t="s">
         <v>564</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="F9" s="13" t="s">
         <v>565</v>
       </c>
-      <c r="F9" s="21" t="s">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
         <v>566</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="B10" s="13" t="s">
+        <v>530</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>567</v>
       </c>
-      <c r="B10" s="21" t="s">
-        <v>530</v>
-      </c>
-      <c r="C10" s="21" t="s">
+      <c r="D10" s="13" t="s">
         <v>568</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="E10" s="13" t="s">
+        <v>529</v>
+      </c>
+      <c r="F10" s="13" t="s">
         <v>569</v>
       </c>
-      <c r="E10" s="21" t="s">
-        <v>529</v>
-      </c>
-      <c r="F10" s="21" t="s">
+    </row>
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
         <v>570</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="s">
+      <c r="B11" s="13" t="s">
         <v>571</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="C11" s="13" t="s">
         <v>572</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="D11" s="13" t="s">
         <v>573</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="E11" s="13" t="s">
         <v>574</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="F11" s="13" t="s">
         <v>575</v>
       </c>
-      <c r="F11" s="21" t="s">
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="B12" s="13" t="s">
         <v>577</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="C12" s="13" t="s">
         <v>578</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="D12" s="13" t="s">
+        <v>573</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>574</v>
+      </c>
+      <c r="F12" s="13" t="s">
         <v>579</v>
       </c>
-      <c r="D12" s="21" t="s">
-        <v>574</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>575</v>
-      </c>
-      <c r="F12" s="21" t="s">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>580</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
+      <c r="B13" s="13" t="s">
         <v>581</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="C13" s="13" t="s">
         <v>582</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="D13" s="13" t="s">
         <v>583</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="E13" s="13" t="s">
         <v>584</v>
       </c>
-      <c r="E13" s="21" t="s">
+      <c r="F13" s="13" t="s">
         <v>585</v>
       </c>
-      <c r="F13" s="21" t="s">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="21" t="s">
+      <c r="B14" s="13" t="s">
         <v>587</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="C14" s="13" t="s">
         <v>588</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="D14" s="13" t="s">
         <v>589</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="E14" s="13" t="s">
         <v>590</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="F14" s="13" t="s">
         <v>591</v>
       </c>
-      <c r="F14" s="21" t="s">
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
         <v>592</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
+      <c r="B15" s="13" t="s">
         <v>593</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="C15" s="13" t="s">
         <v>594</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="D15" s="13" t="s">
         <v>595</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="E15" s="13" t="s">
         <v>596</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="F15" s="13" t="s">
         <v>597</v>
-      </c>
-      <c r="F15" s="21" t="s">
-        <v>598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove the owner's personal name from the workbooks
Owner / prepared-by text, file properties and the saved local file path in
all five workbooks now read "Projento". No rate, rule, duration or score
changed: loader-level model diff shows only settings.info.owner, and
scripts/baseline.mjs is IDENTICAL on 76 scenarios; 763 Vitest cases pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFXWpxLA4sey3e6D3QatTt
</commit_message>
<xml_diff>
--- a/Estates_AI_Programme_v4_3.xlsx
+++ b/Estates_AI_Programme_v4_3.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\estates-ai-tool\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB142D3B-13B6-4D6B-A020-388DED8CE785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2250" yWindow="2250" windowWidth="21600" windowHeight="11295" tabRatio="500" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -1994,7 +1989,7 @@
     <t>Procurement routes follow the RIBA Plan of Work 2020 (11 Oct 2026). New sheet 'Procurement': for each route (PR1 Traditional, PR2 Design &amp; Build 1 Stage, PR3 Design &amp; Build 2 Stage, PR4 Management Contract / Construction Management, matched to the Procurement Reference by ID) the stage after which the contractor is brought in, who does Stage 4, whether the first tender runs alongside Stage 3, and the second-stage price row; and the contract effects (MW: Stages 3–4 replaced by DS34-MW; CDP: client's Stage 4 x 0.8). No overlap of Stage 4 and construction. New Durations rows TN5 (framework direct award), TN7 (second-stage price) and DS34-MW (minor works design and specification).</t>
   </si>
   <si>
-    <t xml:space="preserve">v4.12  ·  October 2026  ·  Nabil Kayali</t>
+    <t xml:space="preserve">v4.12  ·  October 2026  ·  Projento</t>
   </si>
   <si>
     <t xml:space="preserve">Durations checked against eight of the owner's real projects (Oct 2026: Projects A–H — residential, student-residence and academic refurbishments, a demolition, a retail fit-out, a café fit-out, a WC refurbishment and a decarbonisation refurbishment). Handover CH1 cut to 0–3 wks (commissioning runs inside construction; 2 wks on three of the projects). Fit-out CF2 S1–S4 shortened (an 885 m² retail fit-out took 7 wks; a small café about 3 wks). M&amp;E refurb CR1 S1–S2 shortened (a small WC refurbishment: 5 wks). New size band S7 &gt; 10,000 m² with CR1 S7 50–70 (a 17,000 m² occupied student-residence refurbishment: 74 wks planned, forecast about 95). Occupation and phasing uplifts no longer multiply — the higher applies (an occupied 6-section refurbishment: 45 wks). Confirmed unchanged: tender TN1 10–14 (13 wks to award on one project), demolition CD1 (about 14 wks), CR1 S6 (a 3,850 m² full refurbishment: 36 + 6 wks strip-out), planning PL1 (7 wks).</t>

</xml_diff>